<commit_message>
Made some Changes into the Test case Excel File
</commit_message>
<xml_diff>
--- a/testing/Test_Matrix.xlsx
+++ b/testing/Test_Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\10th Session\Apartment Housing Management System\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2336B6F2-9D7B-4BDF-9D50-7E605EA9BF15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7EC7E2-D742-4A87-A3C3-1249F066C782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -305,8 +305,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -614,11 +617,11 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="79.08984375" customWidth="1"/>
-    <col min="4" max="4" width="70.36328125" customWidth="1"/>
-    <col min="5" max="5" width="96" customWidth="1"/>
-    <col min="6" max="6" width="79" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="3" max="3" width="38.81640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="46.26953125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="51.90625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="44.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -628,341 +631,341 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>29</v>
       </c>
       <c r="B6" t="s">
         <v>30</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>35</v>
       </c>
       <c r="B7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>40</v>
       </c>
       <c r="B8" t="s">
         <v>30</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>45</v>
       </c>
       <c r="B9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G9" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>50</v>
       </c>
       <c r="B10" t="s">
         <v>51</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G10" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>56</v>
       </c>
       <c r="B11" t="s">
         <v>51</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="G11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>61</v>
       </c>
       <c r="B12" t="s">
         <v>51</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G12" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>66</v>
       </c>
       <c r="B13" t="s">
         <v>67</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G13" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>72</v>
       </c>
       <c r="B14" t="s">
         <v>67</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G14" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>77</v>
       </c>
       <c r="B15" t="s">
         <v>67</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="1" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed 3 Bugs and Functionality issues
</commit_message>
<xml_diff>
--- a/testing/Test_Matrix.xlsx
+++ b/testing/Test_Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\10th Session\Apartment Housing Management System\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7EC7E2-D742-4A87-A3C3-1249F066C782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E7BF3E-5461-4304-8552-A4C2F6D97E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -276,8 +276,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -305,9 +313,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,25 +637,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>